<commit_message>
Rename interface from Nhà Hàng to Quầy Thuốc and hide tab nav
</commit_message>
<xml_diff>
--- a/tiendumoithang.xlsb.xlsx
+++ b/tiendumoithang.xlsb.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/45df690e3a79b486/hoanglong/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project\Doanhthu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1177" documentId="8_{6648B8AC-EE1D-4AD8-8CC2-896CD253DD6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA2BD139-1CED-438F-88F0-BB05974D7967}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0391600-E606-4881-8E9F-D43EC22DCBCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5200" yWindow="5200" windowWidth="28800" windowHeight="15370" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="thuốc tháng 6.2026" sheetId="26" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="29">
   <si>
     <t>Thời Gian</t>
   </si>
@@ -237,10 +237,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7834,787 +7830,781 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0240CE4D-52DA-480A-BD9F-8F30B29613E4}">
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.90625" style="8" customWidth="1"/>
-    <col min="2" max="3" width="13" style="5" customWidth="1"/>
-    <col min="4" max="5" width="17.36328125" style="5" customWidth="1"/>
-    <col min="6" max="9" width="15.81640625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="14.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" style="5" customWidth="1"/>
+    <col min="4" max="7" width="15.81640625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="14.81640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>46143</v>
       </c>
       <c r="B2" s="5">
         <v>10100</v>
       </c>
+      <c r="C2" s="5">
+        <v>3900</v>
+      </c>
       <c r="D2" s="5">
-        <v>3900</v>
-      </c>
-      <c r="F2" s="5">
         <v>2800</v>
       </c>
-      <c r="G2" s="5">
+      <c r="E2" s="5">
         <v>476</v>
       </c>
-      <c r="J2" s="5">
-        <f>SUM(B2:I2)</f>
+      <c r="H2" s="5">
+        <f>SUM(B2:G2)</f>
         <v>17276</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>46144</v>
       </c>
       <c r="B3" s="5">
         <v>7200</v>
       </c>
+      <c r="C3" s="5">
+        <v>9100</v>
+      </c>
       <c r="D3" s="5">
-        <v>9100</v>
+        <v>5300</v>
+      </c>
+      <c r="E3" s="5">
+        <v>200</v>
       </c>
       <c r="F3" s="5">
-        <v>5300</v>
-      </c>
-      <c r="G3" s="5">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="H3" s="5">
-        <v>600</v>
-      </c>
-      <c r="J3" s="5">
-        <f t="shared" ref="J3:J32" si="0">SUM(B3:I3)</f>
+        <f t="shared" ref="H3:H32" si="0">SUM(B3:G3)</f>
         <v>22400</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>46145</v>
       </c>
       <c r="B4" s="5">
         <v>8000</v>
       </c>
+      <c r="C4" s="5">
+        <v>4600</v>
+      </c>
       <c r="D4" s="5">
-        <v>4600</v>
+        <v>1600</v>
+      </c>
+      <c r="E4" s="5">
+        <v>1300</v>
       </c>
       <c r="F4" s="5">
-        <v>1600</v>
-      </c>
-      <c r="G4" s="5">
-        <v>1300</v>
+        <v>1700</v>
       </c>
       <c r="H4" s="5">
-        <v>1700</v>
-      </c>
-      <c r="J4" s="5">
         <f t="shared" si="0"/>
         <v>17200</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>46146</v>
       </c>
       <c r="B5" s="5">
         <v>8500</v>
       </c>
+      <c r="C5" s="5">
+        <v>6100</v>
+      </c>
       <c r="D5" s="5">
-        <v>6100</v>
+        <v>2600</v>
+      </c>
+      <c r="E5" s="5">
+        <v>1700</v>
       </c>
       <c r="F5" s="5">
-        <v>2600</v>
-      </c>
-      <c r="G5" s="5">
-        <v>1700</v>
+        <v>700</v>
       </c>
       <c r="H5" s="5">
-        <v>700</v>
-      </c>
-      <c r="J5" s="5">
         <f t="shared" si="0"/>
         <v>19600</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>46147</v>
       </c>
       <c r="B6" s="5">
         <v>8200</v>
       </c>
+      <c r="C6" s="5">
+        <v>4400</v>
+      </c>
       <c r="D6" s="5">
-        <v>4400</v>
+        <v>969</v>
+      </c>
+      <c r="E6" s="5">
+        <v>700</v>
       </c>
       <c r="F6" s="5">
-        <v>969</v>
-      </c>
-      <c r="G6" s="5">
-        <v>700</v>
+        <v>130</v>
       </c>
       <c r="H6" s="5">
-        <v>130</v>
-      </c>
-      <c r="J6" s="5">
         <f t="shared" si="0"/>
         <v>14399</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>46148</v>
       </c>
       <c r="B7" s="5">
         <v>10000</v>
       </c>
+      <c r="C7" s="5">
+        <v>3400</v>
+      </c>
       <c r="D7" s="5">
-        <v>3400</v>
+        <v>3300</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1600</v>
       </c>
       <c r="F7" s="5">
-        <v>3300</v>
-      </c>
-      <c r="G7" s="5">
-        <v>1600</v>
+        <v>2600</v>
       </c>
       <c r="H7" s="5">
-        <v>2600</v>
-      </c>
-      <c r="J7" s="5">
         <f t="shared" si="0"/>
         <v>20900</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>46149</v>
       </c>
       <c r="B8" s="5">
         <v>9600</v>
       </c>
+      <c r="C8" s="5">
+        <v>3400</v>
+      </c>
       <c r="D8" s="5">
-        <v>3400</v>
+        <v>2200</v>
+      </c>
+      <c r="E8" s="5">
+        <v>1300</v>
       </c>
       <c r="F8" s="5">
-        <v>2200</v>
-      </c>
-      <c r="G8" s="5">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="H8" s="5">
-        <v>1400</v>
-      </c>
-      <c r="J8" s="5">
         <f t="shared" si="0"/>
         <v>17900</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>46150</v>
       </c>
       <c r="B9" s="5">
         <v>5300</v>
       </c>
+      <c r="C9" s="5">
+        <v>3500</v>
+      </c>
       <c r="D9" s="5">
-        <v>3500</v>
-      </c>
-      <c r="F9" s="5">
         <v>1600</v>
       </c>
-      <c r="G9" s="5">
+      <c r="E9" s="5">
         <v>1000</v>
       </c>
-      <c r="J9" s="5">
+      <c r="H9" s="5">
         <f t="shared" si="0"/>
         <v>11400</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>46151</v>
       </c>
       <c r="B10" s="5">
         <v>6000</v>
       </c>
+      <c r="C10" s="5">
+        <v>5000</v>
+      </c>
       <c r="D10" s="5">
-        <v>5000</v>
+        <v>1300</v>
+      </c>
+      <c r="E10" s="5">
+        <v>3300</v>
       </c>
       <c r="F10" s="5">
-        <v>1300</v>
-      </c>
-      <c r="G10" s="5">
-        <v>3300</v>
+        <v>440</v>
       </c>
       <c r="H10" s="5">
-        <v>440</v>
-      </c>
-      <c r="J10" s="5">
         <f t="shared" si="0"/>
         <v>16040</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46152</v>
       </c>
       <c r="B11" s="5">
         <v>6459</v>
       </c>
+      <c r="C11" s="5">
+        <v>8100</v>
+      </c>
       <c r="D11" s="5">
-        <v>8100</v>
-      </c>
-      <c r="F11" s="5">
         <v>2500</v>
       </c>
-      <c r="G11" s="5">
+      <c r="E11" s="5">
         <v>2500</v>
       </c>
-      <c r="J11" s="5">
+      <c r="H11" s="5">
         <f t="shared" si="0"/>
         <v>19559</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>46153</v>
       </c>
       <c r="B12" s="5">
         <v>4700</v>
       </c>
+      <c r="C12" s="5">
+        <v>3800</v>
+      </c>
       <c r="D12" s="5">
-        <v>3800</v>
+        <v>608</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2416</v>
       </c>
       <c r="F12" s="5">
-        <v>608</v>
-      </c>
-      <c r="G12" s="5">
-        <v>2416</v>
+        <v>8889</v>
       </c>
       <c r="H12" s="5">
-        <v>8889</v>
-      </c>
-      <c r="J12" s="5">
         <f t="shared" si="0"/>
         <v>20413</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>46154</v>
       </c>
       <c r="B13" s="5">
         <v>8600</v>
       </c>
-      <c r="D13" s="5">
+      <c r="C13" s="5">
         <v>3000</v>
       </c>
-      <c r="G13" s="5">
+      <c r="E13" s="5">
         <v>2767</v>
       </c>
+      <c r="F13" s="5">
+        <v>646</v>
+      </c>
       <c r="H13" s="5">
-        <v>646</v>
-      </c>
-      <c r="J13" s="5">
         <f t="shared" si="0"/>
         <v>15013</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>46155</v>
       </c>
       <c r="B14" s="5">
         <v>11050</v>
       </c>
+      <c r="C14" s="5">
+        <v>4650</v>
+      </c>
       <c r="D14" s="5">
-        <v>4650</v>
+        <v>2500</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1483</v>
       </c>
       <c r="F14" s="5">
-        <v>2500</v>
+        <v>85</v>
       </c>
       <c r="G14" s="5">
-        <v>1483</v>
+        <v>1000</v>
       </c>
       <c r="H14" s="5">
-        <v>85</v>
-      </c>
-      <c r="I14" s="5">
-        <v>1000</v>
-      </c>
-      <c r="J14" s="5">
         <f t="shared" si="0"/>
         <v>20768</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>46156</v>
       </c>
       <c r="B15" s="5">
         <v>9600</v>
       </c>
+      <c r="C15" s="5">
+        <v>5700</v>
+      </c>
       <c r="D15" s="5">
-        <v>5700</v>
-      </c>
-      <c r="F15" s="5">
         <v>3700</v>
       </c>
-      <c r="G15" s="5">
+      <c r="E15" s="5">
         <v>254</v>
       </c>
-      <c r="J15" s="5">
+      <c r="H15" s="5">
         <f t="shared" si="0"/>
         <v>19254</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>46157</v>
       </c>
       <c r="B16" s="5">
         <v>7000</v>
       </c>
+      <c r="C16" s="5">
+        <v>4000</v>
+      </c>
       <c r="D16" s="5">
-        <v>4000</v>
+        <v>675</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1100</v>
       </c>
       <c r="F16" s="5">
-        <v>675</v>
-      </c>
-      <c r="G16" s="5">
-        <v>1100</v>
+        <v>750</v>
       </c>
       <c r="H16" s="5">
-        <v>750</v>
-      </c>
-      <c r="J16" s="5">
         <f t="shared" si="0"/>
         <v>13525</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46158</v>
       </c>
       <c r="B17" s="5">
         <v>8000</v>
       </c>
+      <c r="C17" s="5">
+        <v>6500</v>
+      </c>
       <c r="D17" s="5">
-        <v>6500</v>
+        <v>1300</v>
+      </c>
+      <c r="E17" s="5">
+        <v>1400</v>
       </c>
       <c r="F17" s="5">
-        <v>1300</v>
-      </c>
-      <c r="G17" s="5">
-        <v>1400</v>
+        <v>820</v>
       </c>
       <c r="H17" s="5">
-        <v>820</v>
-      </c>
-      <c r="J17" s="5">
         <f t="shared" si="0"/>
         <v>18020</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>46159</v>
       </c>
       <c r="B18" s="5">
         <v>5100</v>
       </c>
+      <c r="C18" s="5">
+        <v>5400</v>
+      </c>
       <c r="D18" s="5">
-        <v>5400</v>
+        <v>1600</v>
+      </c>
+      <c r="E18" s="5">
+        <v>1900</v>
       </c>
       <c r="F18" s="5">
-        <v>1600</v>
-      </c>
-      <c r="G18" s="5">
-        <v>1900</v>
+        <v>1500</v>
       </c>
       <c r="H18" s="5">
-        <v>1500</v>
-      </c>
-      <c r="J18" s="5">
         <f t="shared" si="0"/>
         <v>15500</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>46160</v>
       </c>
       <c r="B19" s="5">
         <v>8500</v>
       </c>
+      <c r="C19" s="5">
+        <v>3800</v>
+      </c>
       <c r="D19" s="5">
-        <v>3800</v>
-      </c>
-      <c r="F19" s="5">
         <v>2800</v>
       </c>
-      <c r="G19" s="5">
+      <c r="E19" s="5">
         <v>882</v>
       </c>
-      <c r="J19" s="5">
+      <c r="H19" s="5">
         <f t="shared" si="0"/>
         <v>15982</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>46161</v>
       </c>
       <c r="B20" s="5">
         <v>5000</v>
       </c>
+      <c r="C20" s="5">
+        <v>5000</v>
+      </c>
       <c r="D20" s="5">
-        <v>5000</v>
+        <v>2000</v>
+      </c>
+      <c r="E20" s="5">
+        <v>1600</v>
       </c>
       <c r="F20" s="5">
-        <v>2000</v>
-      </c>
-      <c r="G20" s="5">
-        <v>1600</v>
+        <v>3800</v>
       </c>
       <c r="H20" s="5">
-        <v>3800</v>
-      </c>
-      <c r="J20" s="5">
         <f t="shared" si="0"/>
         <v>17400</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>46162</v>
       </c>
       <c r="B21" s="5">
         <v>6200</v>
       </c>
+      <c r="C21" s="5">
+        <v>4200</v>
+      </c>
       <c r="D21" s="5">
-        <v>4200</v>
+        <v>1900</v>
+      </c>
+      <c r="E21" s="5">
+        <v>1200</v>
       </c>
       <c r="F21" s="5">
-        <v>1900</v>
-      </c>
-      <c r="G21" s="5">
-        <v>1200</v>
+        <v>490</v>
       </c>
       <c r="H21" s="5">
-        <v>490</v>
-      </c>
-      <c r="J21" s="5">
         <f t="shared" si="0"/>
         <v>13990</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>46163</v>
       </c>
       <c r="B22" s="5">
         <v>4800</v>
       </c>
+      <c r="C22" s="5">
+        <v>5500</v>
+      </c>
       <c r="D22" s="5">
-        <v>5500</v>
+        <v>3800</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
       </c>
       <c r="F22" s="5">
-        <v>3800</v>
-      </c>
-      <c r="G22" s="5">
         <v>0</v>
       </c>
       <c r="H22" s="5">
-        <v>0</v>
-      </c>
-      <c r="J22" s="5">
         <f t="shared" si="0"/>
         <v>14100</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>46164</v>
       </c>
       <c r="B23" s="5">
         <v>5800</v>
       </c>
+      <c r="C23" s="5">
+        <v>4500</v>
+      </c>
       <c r="D23" s="5">
-        <v>4500</v>
+        <v>2100</v>
+      </c>
+      <c r="E23" s="5">
+        <v>200</v>
       </c>
       <c r="F23" s="5">
-        <v>2100</v>
-      </c>
-      <c r="G23" s="5">
-        <v>200</v>
+        <v>1250</v>
       </c>
       <c r="H23" s="5">
-        <v>1250</v>
-      </c>
-      <c r="J23" s="5">
         <f t="shared" si="0"/>
         <v>13850</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46165</v>
       </c>
       <c r="B24" s="5">
         <v>6100</v>
       </c>
+      <c r="C24" s="5">
+        <v>5500</v>
+      </c>
       <c r="D24" s="5">
-        <v>5500</v>
+        <v>2300</v>
+      </c>
+      <c r="E24" s="5">
+        <v>900</v>
       </c>
       <c r="F24" s="5">
-        <v>2300</v>
-      </c>
-      <c r="G24" s="5">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="H24" s="5">
-        <v>1500</v>
-      </c>
-      <c r="J24" s="5">
         <f t="shared" si="0"/>
         <v>16300</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>46166</v>
       </c>
       <c r="B25" s="5">
         <v>7400</v>
       </c>
+      <c r="C25" s="5">
+        <v>3050</v>
+      </c>
       <c r="D25" s="5">
-        <v>3050</v>
+        <v>1200</v>
+      </c>
+      <c r="E25" s="5">
+        <v>750</v>
       </c>
       <c r="F25" s="5">
-        <v>1200</v>
-      </c>
-      <c r="G25" s="5">
-        <v>750</v>
+        <v>450</v>
       </c>
       <c r="H25" s="5">
-        <v>450</v>
-      </c>
-      <c r="J25" s="5">
         <f t="shared" si="0"/>
         <v>12850</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>46167</v>
       </c>
       <c r="B26" s="5">
         <v>10700</v>
       </c>
+      <c r="C26" s="5">
+        <v>4000</v>
+      </c>
       <c r="D26" s="5">
-        <v>4000</v>
+        <v>2100</v>
+      </c>
+      <c r="E26" s="5">
+        <v>500</v>
       </c>
       <c r="F26" s="5">
-        <v>2100</v>
-      </c>
-      <c r="G26" s="5">
-        <v>500</v>
+        <v>2300</v>
       </c>
       <c r="H26" s="5">
-        <v>2300</v>
-      </c>
-      <c r="J26" s="5">
         <f t="shared" si="0"/>
         <v>19600</v>
       </c>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>46168</v>
       </c>
       <c r="B27" s="5">
         <v>5800</v>
       </c>
+      <c r="C27" s="5">
+        <v>5850</v>
+      </c>
       <c r="D27" s="5">
-        <v>5850</v>
+        <v>2000</v>
+      </c>
+      <c r="E27" s="5">
+        <v>850</v>
       </c>
       <c r="F27" s="5">
-        <v>2000</v>
-      </c>
-      <c r="G27" s="5">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="H27" s="5">
-        <v>0</v>
-      </c>
-      <c r="J27" s="5">
         <f t="shared" si="0"/>
         <v>14500</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>46169</v>
       </c>
       <c r="B28" s="5">
         <v>6550</v>
       </c>
+      <c r="C28" s="5">
+        <v>4900</v>
+      </c>
       <c r="D28" s="5">
-        <v>4900</v>
+        <v>2200</v>
+      </c>
+      <c r="E28" s="5">
+        <v>741</v>
       </c>
       <c r="F28" s="5">
-        <v>2200</v>
-      </c>
-      <c r="G28" s="5">
-        <v>741</v>
+        <v>440</v>
       </c>
       <c r="H28" s="5">
-        <v>440</v>
-      </c>
-      <c r="J28" s="5">
         <f t="shared" si="0"/>
         <v>14831</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>46170</v>
       </c>
       <c r="B29" s="5">
         <v>7300</v>
       </c>
+      <c r="C29" s="5">
+        <v>3600</v>
+      </c>
       <c r="D29" s="5">
-        <v>3600</v>
+        <v>3700</v>
+      </c>
+      <c r="E29" s="5">
+        <v>650</v>
       </c>
       <c r="F29" s="5">
-        <v>3700</v>
-      </c>
-      <c r="G29" s="5">
-        <v>650</v>
+        <v>1300</v>
       </c>
       <c r="H29" s="5">
-        <v>1300</v>
-      </c>
-      <c r="J29" s="5">
         <f t="shared" si="0"/>
         <v>16550</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>46171</v>
       </c>
       <c r="B30" s="5">
         <v>7400</v>
       </c>
+      <c r="C30" s="5">
+        <v>5100</v>
+      </c>
       <c r="D30" s="5">
-        <v>5100</v>
+        <v>3900</v>
+      </c>
+      <c r="E30" s="5">
+        <v>323</v>
       </c>
       <c r="F30" s="5">
-        <v>3900</v>
-      </c>
-      <c r="G30" s="5">
-        <v>323</v>
+        <v>477</v>
       </c>
       <c r="H30" s="5">
-        <v>477</v>
-      </c>
-      <c r="J30" s="5">
         <f t="shared" si="0"/>
         <v>17200</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>46172</v>
       </c>
       <c r="B31" s="5">
         <v>6150</v>
       </c>
+      <c r="C31" s="5">
+        <v>6200</v>
+      </c>
       <c r="D31" s="5">
-        <v>6200</v>
+        <v>2900</v>
+      </c>
+      <c r="E31" s="5">
+        <v>1600</v>
       </c>
       <c r="F31" s="5">
-        <v>2900</v>
-      </c>
-      <c r="G31" s="5">
-        <v>1600</v>
+        <v>440</v>
       </c>
       <c r="H31" s="5">
-        <v>440</v>
-      </c>
-      <c r="J31" s="5">
         <f t="shared" si="0"/>
         <v>17290</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>46173</v>
       </c>
       <c r="B32" s="5">
         <v>3550</v>
       </c>
+      <c r="C32" s="5">
+        <v>8450</v>
+      </c>
       <c r="D32" s="5">
-        <v>8450</v>
+        <v>1800</v>
+      </c>
+      <c r="E32" s="5">
+        <v>763</v>
       </c>
       <c r="F32" s="5">
-        <v>1800</v>
-      </c>
-      <c r="G32" s="5">
-        <v>763</v>
+        <v>1100</v>
       </c>
       <c r="H32" s="5">
-        <v>1100</v>
-      </c>
-      <c r="J32" s="5">
         <f t="shared" si="0"/>
         <v>15663</v>
       </c>
     </row>
-    <row r="33" spans="10:13" x14ac:dyDescent="0.35">
-      <c r="J33" s="5">
-        <f>SUM(J2:J32)</f>
+    <row r="33" spans="8:11" x14ac:dyDescent="0.35">
+      <c r="H33" s="5">
+        <f>SUM(H2:H32)</f>
         <v>519273</v>
       </c>
     </row>
-    <row r="34" spans="10:13" x14ac:dyDescent="0.35">
-      <c r="M34" s="5"/>
+    <row r="34" spans="8:11" x14ac:dyDescent="0.35">
+      <c r="K34" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14045,763 +14035,757 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56336ED4-4065-4626-B329-FA78D5C78D67}">
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.90625" style="8" customWidth="1"/>
-    <col min="2" max="3" width="13" style="5" customWidth="1"/>
-    <col min="4" max="5" width="17.36328125" style="5" customWidth="1"/>
-    <col min="6" max="9" width="15.81640625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="14.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" style="5" customWidth="1"/>
+    <col min="4" max="7" width="15.81640625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="14.81640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>46113</v>
       </c>
+      <c r="B2" s="5">
+        <v>10000</v>
+      </c>
       <c r="C2" s="5">
-        <v>10000</v>
+        <v>6250</v>
+      </c>
+      <c r="D2" s="5">
+        <v>3800</v>
       </c>
       <c r="E2" s="5">
-        <v>6250</v>
-      </c>
-      <c r="F2" s="5">
-        <v>3800</v>
-      </c>
-      <c r="G2" s="5">
         <v>320</v>
       </c>
-      <c r="J2" s="5">
-        <f>SUM(B2:I2)</f>
+      <c r="H2" s="5">
+        <f>SUM(B2:G2)</f>
         <v>20370</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>46114</v>
       </c>
+      <c r="B3" s="5">
+        <v>11900</v>
+      </c>
       <c r="C3" s="5">
-        <v>11900</v>
+        <v>5000</v>
+      </c>
+      <c r="D3" s="5">
+        <v>2800</v>
       </c>
       <c r="E3" s="5">
-        <v>5000</v>
-      </c>
-      <c r="F3" s="5">
-        <v>2800</v>
-      </c>
-      <c r="G3" s="5">
         <v>2300</v>
       </c>
-      <c r="J3" s="5">
-        <f t="shared" ref="J3:J31" si="0">SUM(B3:I3)</f>
+      <c r="H3" s="5">
+        <f>SUM(B3:G3)</f>
         <v>22000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>46115</v>
       </c>
+      <c r="B4" s="5">
+        <v>9900</v>
+      </c>
       <c r="C4" s="5">
-        <v>9900</v>
+        <v>2800</v>
+      </c>
+      <c r="D4" s="5">
+        <v>5000</v>
       </c>
       <c r="E4" s="5">
-        <v>2800</v>
+        <v>720</v>
       </c>
       <c r="F4" s="5">
-        <v>5000</v>
-      </c>
-      <c r="G4" s="5">
-        <v>720</v>
+        <v>7600</v>
       </c>
       <c r="H4" s="5">
-        <v>7600</v>
-      </c>
-      <c r="J4" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B4:G4)</f>
         <v>26020</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>46116</v>
       </c>
+      <c r="B5" s="5">
+        <v>8100</v>
+      </c>
       <c r="C5" s="5">
-        <v>8100</v>
+        <v>5000</v>
+      </c>
+      <c r="D5" s="5">
+        <v>2700</v>
       </c>
       <c r="E5" s="5">
-        <v>5000</v>
-      </c>
-      <c r="F5" s="5">
-        <v>2700</v>
-      </c>
-      <c r="G5" s="5">
         <v>274</v>
       </c>
-      <c r="J5" s="5">
-        <f t="shared" si="0"/>
+      <c r="H5" s="5">
+        <f>SUM(B5:G5)</f>
         <v>16074</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>46117</v>
       </c>
+      <c r="B6" s="5">
+        <v>8400</v>
+      </c>
       <c r="C6" s="5">
-        <v>8400</v>
+        <v>7800</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1300</v>
       </c>
       <c r="E6" s="5">
-        <v>7800</v>
+        <v>2200</v>
       </c>
       <c r="F6" s="5">
-        <v>1300</v>
-      </c>
-      <c r="G6" s="5">
-        <v>2200</v>
+        <v>754</v>
       </c>
       <c r="H6" s="5">
-        <v>754</v>
-      </c>
-      <c r="J6" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B6:G6)</f>
         <v>20454</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>46118</v>
       </c>
+      <c r="B7" s="5">
+        <v>8900</v>
+      </c>
       <c r="C7" s="5">
-        <v>8900</v>
+        <v>7400</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1700</v>
       </c>
       <c r="E7" s="5">
-        <v>7400</v>
+        <v>2100</v>
       </c>
       <c r="F7" s="5">
-        <v>1700</v>
-      </c>
-      <c r="G7" s="5">
-        <v>2100</v>
+        <v>235</v>
       </c>
       <c r="H7" s="5">
-        <v>235</v>
-      </c>
-      <c r="J7" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B7:G7)</f>
         <v>20335</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>46119</v>
       </c>
+      <c r="B8" s="5">
+        <v>9225</v>
+      </c>
       <c r="C8" s="5">
-        <v>9225</v>
+        <v>5900</v>
+      </c>
+      <c r="D8" s="5">
+        <v>2300</v>
       </c>
       <c r="E8" s="5">
-        <v>5900</v>
+        <v>1400</v>
       </c>
       <c r="F8" s="5">
-        <v>2300</v>
-      </c>
-      <c r="G8" s="5">
-        <v>1400</v>
+        <v>170</v>
       </c>
       <c r="H8" s="5">
-        <v>170</v>
-      </c>
-      <c r="J8" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B8:G8)</f>
         <v>18995</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>46120</v>
       </c>
+      <c r="B9" s="5">
+        <v>8500</v>
+      </c>
       <c r="C9" s="5">
-        <v>8500</v>
+        <v>5500</v>
+      </c>
+      <c r="D9" s="5">
+        <v>2000</v>
       </c>
       <c r="E9" s="5">
-        <v>5500</v>
+        <v>908</v>
       </c>
       <c r="F9" s="5">
-        <v>2000</v>
-      </c>
-      <c r="G9" s="5">
-        <v>908</v>
+        <v>280</v>
       </c>
       <c r="H9" s="5">
-        <v>280</v>
-      </c>
-      <c r="J9" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B9:G9)</f>
         <v>17188</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>46121</v>
       </c>
+      <c r="B10" s="5">
+        <v>11200</v>
+      </c>
       <c r="C10" s="5">
-        <v>11200</v>
+        <v>6400</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1400</v>
       </c>
       <c r="E10" s="5">
-        <v>6400</v>
+        <v>1500</v>
       </c>
       <c r="F10" s="5">
-        <v>1400</v>
-      </c>
-      <c r="G10" s="5">
-        <v>1500</v>
+        <v>3600</v>
       </c>
       <c r="H10" s="5">
-        <v>3600</v>
-      </c>
-      <c r="J10" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B10:G10)</f>
         <v>24100</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46122</v>
       </c>
+      <c r="B11" s="5">
+        <v>6080</v>
+      </c>
       <c r="C11" s="5">
-        <v>6080</v>
+        <v>7650</v>
+      </c>
+      <c r="D11" s="5">
+        <v>3300</v>
       </c>
       <c r="E11" s="5">
-        <v>7650</v>
+        <v>763</v>
       </c>
       <c r="F11" s="5">
-        <v>3300</v>
-      </c>
-      <c r="G11" s="5">
-        <v>763</v>
+        <v>1900</v>
       </c>
       <c r="H11" s="5">
-        <v>1900</v>
-      </c>
-      <c r="J11" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B11:G11)</f>
         <v>19693</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>46123</v>
       </c>
+      <c r="B12" s="5">
+        <v>12850</v>
+      </c>
       <c r="C12" s="5">
-        <v>12850</v>
+        <v>6400</v>
+      </c>
+      <c r="D12" s="5">
+        <v>2000</v>
       </c>
       <c r="E12" s="5">
-        <v>6400</v>
+        <v>800</v>
       </c>
       <c r="F12" s="5">
-        <v>2000</v>
-      </c>
-      <c r="G12" s="5">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="H12" s="5">
-        <v>600</v>
-      </c>
-      <c r="J12" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B12:G12)</f>
         <v>22650</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>46124</v>
       </c>
+      <c r="B13" s="5">
+        <v>5000</v>
+      </c>
       <c r="C13" s="5">
-        <v>5000</v>
+        <v>8000</v>
+      </c>
+      <c r="D13" s="5">
+        <v>2400</v>
       </c>
       <c r="E13" s="5">
-        <v>8000</v>
+        <v>1100</v>
       </c>
       <c r="F13" s="5">
-        <v>2400</v>
-      </c>
-      <c r="G13" s="5">
-        <v>1100</v>
+        <v>1500</v>
       </c>
       <c r="H13" s="5">
-        <v>1500</v>
-      </c>
-      <c r="J13" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B13:G13)</f>
         <v>18000</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>46125</v>
       </c>
+      <c r="B14" s="5">
+        <v>6600</v>
+      </c>
       <c r="C14" s="5">
-        <v>6600</v>
+        <v>7100</v>
+      </c>
+      <c r="D14" s="5">
+        <v>2600</v>
       </c>
       <c r="E14" s="5">
-        <v>7100</v>
-      </c>
-      <c r="F14" s="5">
-        <v>2600</v>
-      </c>
-      <c r="G14" s="5">
         <v>1100</v>
       </c>
-      <c r="J14" s="5">
-        <f t="shared" si="0"/>
+      <c r="H14" s="5">
+        <f>SUM(B14:G14)</f>
         <v>17400</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>46126</v>
       </c>
+      <c r="B15" s="5">
+        <v>7100</v>
+      </c>
       <c r="C15" s="5">
-        <v>7100</v>
+        <v>4500</v>
+      </c>
+      <c r="D15" s="5">
+        <v>2400</v>
       </c>
       <c r="E15" s="5">
-        <v>4500</v>
+        <v>1300</v>
       </c>
       <c r="F15" s="5">
-        <v>2400</v>
-      </c>
-      <c r="G15" s="5">
-        <v>1300</v>
+        <v>1400</v>
       </c>
       <c r="H15" s="5">
-        <v>1400</v>
-      </c>
-      <c r="J15" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B15:G15)</f>
         <v>16700</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>46127</v>
       </c>
+      <c r="B16" s="5">
+        <v>9100</v>
+      </c>
       <c r="C16" s="5">
-        <v>9100</v>
+        <v>4500</v>
+      </c>
+      <c r="D16" s="5">
+        <v>2600</v>
       </c>
       <c r="E16" s="5">
-        <v>4500</v>
+        <v>1100</v>
       </c>
       <c r="F16" s="5">
-        <v>2600</v>
+        <v>1400</v>
       </c>
       <c r="G16" s="5">
-        <v>1100</v>
+        <v>2500</v>
       </c>
       <c r="H16" s="5">
-        <v>1400</v>
-      </c>
-      <c r="I16" s="5">
-        <v>2500</v>
-      </c>
-      <c r="J16" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B16:G16)</f>
         <v>21200</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46128</v>
       </c>
+      <c r="B17" s="5">
+        <v>10000</v>
+      </c>
       <c r="C17" s="5">
-        <v>10000</v>
+        <v>4900</v>
+      </c>
+      <c r="D17" s="5">
+        <v>2600</v>
       </c>
       <c r="E17" s="5">
-        <v>4900</v>
+        <v>120</v>
       </c>
       <c r="F17" s="5">
-        <v>2600</v>
-      </c>
-      <c r="G17" s="5">
-        <v>120</v>
+        <v>925</v>
       </c>
       <c r="H17" s="5">
-        <v>925</v>
-      </c>
-      <c r="J17" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B17:G17)</f>
         <v>18545</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>46129</v>
       </c>
+      <c r="B18" s="5">
+        <v>6900</v>
+      </c>
       <c r="C18" s="5">
         <v>6900</v>
       </c>
+      <c r="D18" s="5">
+        <v>3000</v>
+      </c>
       <c r="E18" s="5">
-        <v>6900</v>
+        <v>755</v>
       </c>
       <c r="F18" s="5">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="G18" s="5">
-        <v>755</v>
+        <v>1000</v>
       </c>
       <c r="H18" s="5">
-        <v>1000</v>
-      </c>
-      <c r="I18" s="5">
-        <v>1000</v>
-      </c>
-      <c r="J18" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B18:G18)</f>
         <v>19555</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>46130</v>
       </c>
+      <c r="B19" s="5">
+        <v>5500</v>
+      </c>
       <c r="C19" s="5">
-        <v>5500</v>
+        <v>4550</v>
+      </c>
+      <c r="D19" s="5">
+        <v>3200</v>
       </c>
       <c r="E19" s="5">
-        <v>4550</v>
-      </c>
-      <c r="F19" s="5">
-        <v>3200</v>
+        <v>500</v>
       </c>
       <c r="G19" s="5">
-        <v>500</v>
-      </c>
-      <c r="I19" s="5">
         <v>2242</v>
       </c>
-      <c r="J19" s="5">
-        <f t="shared" si="0"/>
+      <c r="H19" s="5">
+        <f>SUM(B19:G19)</f>
         <v>15992</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>46131</v>
       </c>
+      <c r="B20" s="5">
+        <v>5800</v>
+      </c>
       <c r="C20" s="5">
-        <v>5800</v>
+        <v>6700</v>
+      </c>
+      <c r="D20" s="5">
+        <v>2600</v>
       </c>
       <c r="E20" s="5">
-        <v>6700</v>
+        <v>2000</v>
       </c>
       <c r="F20" s="5">
-        <v>2600</v>
-      </c>
-      <c r="G20" s="5">
-        <v>2000</v>
+        <v>240</v>
       </c>
       <c r="H20" s="5">
-        <v>240</v>
-      </c>
-      <c r="J20" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B20:G20)</f>
         <v>17340</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>46132</v>
       </c>
+      <c r="B21" s="5">
+        <v>4300</v>
+      </c>
       <c r="C21" s="5">
-        <v>4300</v>
+        <v>10000</v>
+      </c>
+      <c r="D21" s="5">
+        <v>3000</v>
       </c>
       <c r="E21" s="5">
-        <v>10000</v>
+        <v>1200</v>
       </c>
       <c r="F21" s="5">
-        <v>3000</v>
+        <v>1200</v>
       </c>
       <c r="G21" s="5">
-        <v>1200</v>
+        <v>2200</v>
       </c>
       <c r="H21" s="5">
-        <v>1200</v>
-      </c>
-      <c r="I21" s="5">
-        <v>2200</v>
-      </c>
-      <c r="J21" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B21:G21)</f>
         <v>21900</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>46133</v>
       </c>
+      <c r="B22" s="5">
+        <v>9900</v>
+      </c>
       <c r="C22" s="5">
-        <v>9900</v>
+        <v>5500</v>
+      </c>
+      <c r="D22" s="5">
+        <v>209</v>
       </c>
       <c r="E22" s="5">
-        <v>5500</v>
+        <v>3300</v>
       </c>
       <c r="F22" s="5">
-        <v>209</v>
-      </c>
-      <c r="G22" s="5">
-        <v>3300</v>
+        <v>150</v>
       </c>
       <c r="H22" s="5">
-        <v>150</v>
-      </c>
-      <c r="J22" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B22:G22)</f>
         <v>19059</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>46134</v>
       </c>
+      <c r="B23" s="5">
+        <v>8600</v>
+      </c>
       <c r="C23" s="5">
-        <v>8600</v>
+        <v>4650</v>
+      </c>
+      <c r="D23" s="5">
+        <v>780</v>
       </c>
       <c r="E23" s="5">
-        <v>4650</v>
+        <v>6600</v>
       </c>
       <c r="F23" s="5">
-        <v>780</v>
-      </c>
-      <c r="G23" s="5">
-        <v>6600</v>
+        <v>100</v>
       </c>
       <c r="H23" s="5">
-        <v>100</v>
-      </c>
-      <c r="J23" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B23:G23)</f>
         <v>20730</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46135</v>
       </c>
+      <c r="B24" s="5">
+        <v>11200</v>
+      </c>
       <c r="C24" s="5">
-        <v>11200</v>
+        <v>7600</v>
+      </c>
+      <c r="D24" s="5">
+        <v>935</v>
       </c>
       <c r="E24" s="5">
-        <v>7600</v>
-      </c>
-      <c r="F24" s="5">
-        <v>935</v>
-      </c>
-      <c r="G24" s="5">
         <v>3400</v>
       </c>
-      <c r="J24" s="5">
-        <f t="shared" si="0"/>
+      <c r="H24" s="5">
+        <f>SUM(B24:G24)</f>
         <v>23135</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>46136</v>
       </c>
+      <c r="B25" s="5">
+        <v>6800</v>
+      </c>
       <c r="C25" s="5">
-        <v>6800</v>
+        <v>7500</v>
+      </c>
+      <c r="D25" s="5">
+        <v>745</v>
       </c>
       <c r="E25" s="5">
-        <v>7500</v>
+        <v>3900</v>
       </c>
       <c r="F25" s="5">
-        <v>745</v>
-      </c>
-      <c r="G25" s="5">
-        <v>3900</v>
+        <v>555</v>
       </c>
       <c r="H25" s="5">
-        <v>555</v>
-      </c>
-      <c r="J25" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B25:G25)</f>
         <v>19500</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>46137</v>
       </c>
+      <c r="B26" s="5">
+        <v>6700</v>
+      </c>
       <c r="C26" s="5">
-        <v>6700</v>
+        <v>5700</v>
+      </c>
+      <c r="D26" s="5">
+        <v>130</v>
       </c>
       <c r="E26" s="5">
-        <v>5700</v>
+        <v>3900</v>
       </c>
       <c r="F26" s="5">
-        <v>130</v>
-      </c>
-      <c r="G26" s="5">
-        <v>3900</v>
+        <v>750</v>
       </c>
       <c r="H26" s="5">
-        <v>750</v>
-      </c>
-      <c r="J26" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B26:G26)</f>
         <v>17180</v>
       </c>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>46138</v>
       </c>
+      <c r="C27" s="5">
+        <v>7200</v>
+      </c>
+      <c r="D27" s="5">
+        <v>343</v>
+      </c>
       <c r="E27" s="5">
-        <v>7200</v>
+        <v>1700</v>
       </c>
       <c r="F27" s="5">
-        <v>343</v>
-      </c>
-      <c r="G27" s="5">
-        <v>1700</v>
+        <v>450</v>
       </c>
       <c r="H27" s="5">
-        <v>450</v>
-      </c>
-      <c r="J27" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B27:G27)</f>
         <v>9693</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>46139</v>
       </c>
+      <c r="B28" s="5">
+        <v>5200</v>
+      </c>
       <c r="C28" s="5">
-        <v>5200</v>
+        <v>6700</v>
+      </c>
+      <c r="D28" s="5">
+        <v>544</v>
       </c>
       <c r="E28" s="5">
-        <v>6700</v>
+        <v>4800</v>
       </c>
       <c r="F28" s="5">
-        <v>544</v>
-      </c>
-      <c r="G28" s="5">
-        <v>4800</v>
+        <v>830</v>
       </c>
       <c r="H28" s="5">
-        <v>830</v>
-      </c>
-      <c r="J28" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B28:G28)</f>
         <v>18074</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>46140</v>
       </c>
+      <c r="B29" s="5">
+        <v>8700</v>
+      </c>
       <c r="C29" s="5">
-        <v>8700</v>
+        <v>6900</v>
+      </c>
+      <c r="D29" s="5">
+        <v>2700</v>
       </c>
       <c r="E29" s="5">
-        <v>6900</v>
+        <v>1500</v>
       </c>
       <c r="F29" s="5">
-        <v>2700</v>
-      </c>
-      <c r="G29" s="5">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="H29" s="5">
-        <v>200</v>
-      </c>
-      <c r="J29" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B29:G29)</f>
         <v>20000</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>46141</v>
       </c>
+      <c r="B30" s="5">
+        <v>5900</v>
+      </c>
       <c r="C30" s="5">
-        <v>5900</v>
+        <v>8521</v>
+      </c>
+      <c r="D30" s="5">
+        <v>4400</v>
       </c>
       <c r="E30" s="5">
-        <v>8521</v>
-      </c>
-      <c r="F30" s="5">
-        <v>4400</v>
-      </c>
-      <c r="G30" s="5">
         <v>500</v>
       </c>
-      <c r="J30" s="5">
-        <f t="shared" si="0"/>
+      <c r="H30" s="5">
+        <f>SUM(B30:G30)</f>
         <v>19321</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>46142</v>
       </c>
+      <c r="B31" s="5">
+        <v>3900</v>
+      </c>
       <c r="C31" s="5">
-        <v>3900</v>
+        <v>7500</v>
+      </c>
+      <c r="D31" s="5">
+        <v>976</v>
       </c>
       <c r="E31" s="5">
-        <v>7500</v>
-      </c>
-      <c r="F31" s="5">
-        <v>976</v>
-      </c>
-      <c r="G31" s="5">
         <v>226</v>
       </c>
-      <c r="J31" s="5">
-        <f t="shared" si="0"/>
+      <c r="H31" s="5">
+        <f>SUM(B31:G31)</f>
         <v>12602</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="J32" s="5">
-        <f>SUM(J2:J31)</f>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H32" s="5">
+        <f>SUM(H2:H31)</f>
         <v>573805</v>
       </c>
     </row>
-    <row r="34" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M34" s="5"/>
+    <row r="34" spans="11:11" x14ac:dyDescent="0.35">
+      <c r="K34" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14811,610 +14795,604 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B288AB05-C68B-4A6B-93AA-0988A6FCEFD0}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.90625" style="8" customWidth="1"/>
-    <col min="2" max="3" width="13" style="5" customWidth="1"/>
-    <col min="4" max="5" width="17.36328125" style="5" customWidth="1"/>
-    <col min="6" max="7" width="15.81640625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="14.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="15.81640625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>46082</v>
       </c>
       <c r="B2" s="5">
         <v>9500</v>
       </c>
+      <c r="C2" s="5">
+        <v>5700</v>
+      </c>
       <c r="D2" s="5">
-        <v>5700</v>
+        <v>5400</v>
       </c>
       <c r="F2" s="5">
-        <v>5400</v>
-      </c>
-      <c r="H2" s="5">
-        <f>SUM(B2:G2)</f>
+        <f>SUM(B2:E2)</f>
         <v>20600</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>46083</v>
       </c>
       <c r="B3" s="5">
         <v>5000</v>
       </c>
+      <c r="C3" s="5">
+        <v>8648</v>
+      </c>
       <c r="D3" s="5">
-        <v>8648</v>
+        <v>4500</v>
       </c>
       <c r="F3" s="5">
-        <v>4500</v>
-      </c>
-      <c r="H3" s="5">
-        <f t="shared" ref="H3:H32" si="0">SUM(B3:G3)</f>
+        <f t="shared" ref="F3:F32" si="0">SUM(B3:E3)</f>
         <v>18148</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>46084</v>
       </c>
       <c r="B4" s="5">
         <v>11076</v>
       </c>
+      <c r="C4" s="5">
+        <v>6100</v>
+      </c>
       <c r="D4" s="5">
-        <v>6100</v>
+        <v>4100</v>
       </c>
       <c r="F4" s="5">
-        <v>4100</v>
-      </c>
-      <c r="H4" s="5">
         <f t="shared" si="0"/>
         <v>21276</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>46085</v>
       </c>
       <c r="B5" s="5">
         <v>5200</v>
       </c>
+      <c r="C5" s="5">
+        <v>11900</v>
+      </c>
       <c r="D5" s="5">
-        <v>11900</v>
+        <v>2800</v>
       </c>
       <c r="F5" s="5">
-        <v>2800</v>
-      </c>
-      <c r="H5" s="5">
         <f t="shared" si="0"/>
         <v>19900</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>46086</v>
       </c>
       <c r="B6" s="5">
         <v>14600</v>
       </c>
+      <c r="C6" s="5">
+        <v>7700</v>
+      </c>
       <c r="D6" s="5">
-        <v>7700</v>
+        <v>6200</v>
       </c>
       <c r="F6" s="5">
-        <v>6200</v>
-      </c>
-      <c r="H6" s="5">
         <f t="shared" si="0"/>
         <v>28500</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>46087</v>
       </c>
       <c r="B7" s="5">
         <v>13500</v>
       </c>
+      <c r="C7" s="5">
+        <v>4000</v>
+      </c>
       <c r="D7" s="5">
-        <v>4000</v>
+        <v>9900</v>
       </c>
       <c r="F7" s="5">
-        <v>9900</v>
-      </c>
-      <c r="H7" s="5">
         <f t="shared" si="0"/>
         <v>27400</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>46088</v>
       </c>
       <c r="B8" s="5">
         <v>8600</v>
       </c>
+      <c r="C8" s="5">
+        <v>4900</v>
+      </c>
       <c r="D8" s="5">
-        <v>4900</v>
+        <v>5100</v>
       </c>
       <c r="F8" s="5">
-        <v>5100</v>
-      </c>
-      <c r="H8" s="5">
         <f t="shared" si="0"/>
         <v>18600</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>46089</v>
       </c>
       <c r="B9" s="5">
         <v>11200</v>
       </c>
+      <c r="C9" s="5">
+        <v>4200</v>
+      </c>
       <c r="D9" s="5">
-        <v>4200</v>
+        <v>3800</v>
       </c>
       <c r="F9" s="5">
-        <v>3800</v>
-      </c>
-      <c r="H9" s="5">
         <f t="shared" si="0"/>
         <v>19200</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>46090</v>
       </c>
       <c r="B10" s="5">
         <v>3600</v>
       </c>
+      <c r="C10" s="5">
+        <v>12300</v>
+      </c>
       <c r="D10" s="5">
-        <v>12300</v>
+        <v>5900</v>
       </c>
       <c r="F10" s="5">
-        <v>5900</v>
-      </c>
-      <c r="H10" s="5">
         <f t="shared" si="0"/>
         <v>21800</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46091</v>
       </c>
       <c r="B11" s="5">
         <v>8950</v>
       </c>
+      <c r="C11" s="5">
+        <v>4600</v>
+      </c>
       <c r="D11" s="5">
-        <v>4600</v>
+        <v>6200</v>
       </c>
       <c r="F11" s="5">
-        <v>6200</v>
-      </c>
-      <c r="H11" s="5">
         <f t="shared" si="0"/>
         <v>19750</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>46092</v>
       </c>
       <c r="B12" s="5">
         <v>9700</v>
       </c>
+      <c r="C12" s="5">
+        <v>5300</v>
+      </c>
       <c r="D12" s="5">
-        <v>5300</v>
+        <v>4000</v>
       </c>
       <c r="F12" s="5">
-        <v>4000</v>
-      </c>
-      <c r="H12" s="5">
         <f t="shared" si="0"/>
         <v>19000</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>46093</v>
       </c>
       <c r="B13" s="5">
         <v>8600</v>
       </c>
+      <c r="C13" s="5">
+        <v>5400</v>
+      </c>
       <c r="D13" s="5">
-        <v>5400</v>
+        <v>3600</v>
       </c>
       <c r="F13" s="5">
-        <v>3600</v>
-      </c>
-      <c r="H13" s="5">
         <f t="shared" si="0"/>
         <v>17600</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>46094</v>
       </c>
       <c r="B14" s="5">
         <v>7700</v>
       </c>
+      <c r="C14" s="5">
+        <v>7400</v>
+      </c>
       <c r="D14" s="5">
-        <v>7400</v>
+        <v>2900</v>
       </c>
       <c r="F14" s="5">
-        <v>2900</v>
-      </c>
-      <c r="H14" s="5">
         <f t="shared" si="0"/>
         <v>18000</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>46095</v>
       </c>
       <c r="B15" s="5">
         <v>5800</v>
       </c>
+      <c r="C15" s="5">
+        <v>3400</v>
+      </c>
       <c r="D15" s="5">
-        <v>3400</v>
+        <v>1600</v>
       </c>
       <c r="F15" s="5">
-        <v>1600</v>
-      </c>
-      <c r="H15" s="5">
         <f t="shared" si="0"/>
         <v>10800</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>46096</v>
       </c>
       <c r="B16" s="5">
         <v>12500</v>
       </c>
+      <c r="C16" s="5">
+        <v>2800</v>
+      </c>
       <c r="D16" s="5">
-        <v>2800</v>
+        <v>5700</v>
       </c>
       <c r="F16" s="5">
-        <v>5700</v>
-      </c>
-      <c r="H16" s="5">
         <f t="shared" si="0"/>
         <v>21000</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46097</v>
       </c>
       <c r="B17" s="5">
         <v>12200</v>
       </c>
+      <c r="C17" s="5">
+        <v>5100</v>
+      </c>
       <c r="D17" s="5">
-        <v>5100</v>
+        <v>5300</v>
       </c>
       <c r="F17" s="5">
-        <v>5300</v>
-      </c>
-      <c r="H17" s="5">
         <f t="shared" si="0"/>
         <v>22600</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>46098</v>
       </c>
       <c r="B18" s="5">
         <v>7200</v>
       </c>
+      <c r="C18" s="5">
+        <v>6500</v>
+      </c>
       <c r="D18" s="5">
-        <v>6500</v>
+        <v>5500</v>
       </c>
       <c r="F18" s="5">
-        <v>5500</v>
-      </c>
-      <c r="H18" s="5">
         <f t="shared" si="0"/>
         <v>19200</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>46099</v>
       </c>
       <c r="B19" s="5">
         <v>8700</v>
       </c>
+      <c r="C19" s="5">
+        <v>4000</v>
+      </c>
       <c r="D19" s="5">
-        <v>4000</v>
+        <v>6800</v>
       </c>
       <c r="F19" s="5">
-        <v>6800</v>
-      </c>
-      <c r="H19" s="5">
         <f t="shared" si="0"/>
         <v>19500</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>46100</v>
       </c>
       <c r="B20" s="5">
         <v>5700</v>
       </c>
+      <c r="C20" s="5">
+        <v>4200</v>
+      </c>
       <c r="D20" s="5">
-        <v>4200</v>
+        <v>3200</v>
       </c>
       <c r="F20" s="5">
-        <v>3200</v>
-      </c>
-      <c r="H20" s="5">
         <f t="shared" si="0"/>
         <v>13100</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>46101</v>
       </c>
       <c r="B21" s="5">
         <v>9400</v>
       </c>
+      <c r="C21" s="5">
+        <v>5000</v>
+      </c>
       <c r="D21" s="5">
-        <v>5000</v>
+        <v>3600</v>
       </c>
       <c r="F21" s="5">
-        <v>3600</v>
-      </c>
-      <c r="H21" s="5">
         <f t="shared" si="0"/>
         <v>18000</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>46102</v>
       </c>
       <c r="B22" s="5">
         <v>7800</v>
       </c>
+      <c r="C22" s="5">
+        <v>6300</v>
+      </c>
       <c r="D22" s="5">
-        <v>6300</v>
+        <v>3500</v>
       </c>
       <c r="F22" s="5">
-        <v>3500</v>
-      </c>
-      <c r="H22" s="5">
         <f t="shared" si="0"/>
         <v>17600</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>46103</v>
       </c>
       <c r="B23" s="5">
         <v>7600</v>
       </c>
+      <c r="C23" s="5">
+        <v>5500</v>
+      </c>
       <c r="D23" s="5">
-        <v>5500</v>
+        <v>2500</v>
       </c>
       <c r="F23" s="5">
-        <v>2500</v>
-      </c>
-      <c r="H23" s="5">
         <f t="shared" si="0"/>
         <v>15600</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46104</v>
       </c>
       <c r="B24" s="5">
         <v>8500</v>
       </c>
+      <c r="C24" s="5">
+        <v>7100</v>
+      </c>
       <c r="D24" s="5">
-        <v>7100</v>
+        <v>9000</v>
       </c>
       <c r="F24" s="5">
-        <v>9000</v>
-      </c>
-      <c r="H24" s="5">
         <f t="shared" si="0"/>
         <v>24600</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>46105</v>
       </c>
       <c r="B25" s="5">
         <v>12000</v>
       </c>
+      <c r="C25" s="5">
+        <v>5400</v>
+      </c>
       <c r="D25" s="5">
-        <v>5400</v>
+        <v>4580</v>
       </c>
       <c r="F25" s="5">
-        <v>4580</v>
-      </c>
-      <c r="H25" s="5">
         <f t="shared" si="0"/>
         <v>21980</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>46106</v>
       </c>
       <c r="B26" s="5">
         <v>9281</v>
       </c>
+      <c r="C26" s="5">
+        <v>3850</v>
+      </c>
       <c r="D26" s="5">
-        <v>3850</v>
+        <v>5500</v>
       </c>
       <c r="F26" s="5">
-        <v>5500</v>
-      </c>
-      <c r="H26" s="5">
         <f t="shared" si="0"/>
         <v>18631</v>
       </c>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>46107</v>
       </c>
       <c r="B27" s="5">
         <v>5900</v>
       </c>
+      <c r="C27" s="5">
+        <v>3400</v>
+      </c>
       <c r="D27" s="5">
-        <v>3400</v>
+        <v>4200</v>
       </c>
       <c r="F27" s="5">
-        <v>4200</v>
-      </c>
-      <c r="H27" s="5">
         <f t="shared" si="0"/>
         <v>13500</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>46108</v>
       </c>
       <c r="B28" s="5">
         <v>10700</v>
       </c>
+      <c r="C28" s="5">
+        <v>6400</v>
+      </c>
       <c r="D28" s="5">
-        <v>6400</v>
+        <v>6000</v>
       </c>
       <c r="F28" s="5">
-        <v>6000</v>
-      </c>
-      <c r="H28" s="5">
         <f t="shared" si="0"/>
         <v>23100</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>46109</v>
       </c>
       <c r="B29" s="5">
         <v>7800</v>
       </c>
+      <c r="C29" s="5">
+        <v>3500</v>
+      </c>
       <c r="D29" s="5">
-        <v>3500</v>
+        <v>6200</v>
       </c>
       <c r="F29" s="5">
-        <v>6200</v>
-      </c>
-      <c r="H29" s="5">
         <f t="shared" si="0"/>
         <v>17500</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>46110</v>
       </c>
       <c r="B30" s="5">
         <v>9800</v>
       </c>
+      <c r="C30" s="5">
+        <v>9300</v>
+      </c>
       <c r="D30" s="5">
-        <v>9300</v>
+        <v>4000</v>
       </c>
       <c r="F30" s="5">
-        <v>4000</v>
-      </c>
-      <c r="H30" s="5">
         <f t="shared" si="0"/>
         <v>23100</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>46111</v>
       </c>
       <c r="B31" s="5">
         <v>7122</v>
       </c>
+      <c r="C31" s="5">
+        <v>4700</v>
+      </c>
       <c r="D31" s="5">
-        <v>4700</v>
+        <v>1800</v>
       </c>
       <c r="F31" s="5">
-        <v>1800</v>
-      </c>
-      <c r="H31" s="5">
         <f t="shared" si="0"/>
         <v>13622</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>46112</v>
       </c>
       <c r="B32" s="5">
         <v>6500</v>
       </c>
+      <c r="C32" s="5">
+        <v>3600</v>
+      </c>
       <c r="D32" s="5">
-        <v>3600</v>
+        <v>6600</v>
       </c>
       <c r="F32" s="5">
-        <v>6600</v>
-      </c>
-      <c r="H32" s="5">
         <f t="shared" si="0"/>
         <v>16700</v>
       </c>
     </row>
-    <row r="33" spans="8:11" x14ac:dyDescent="0.35">
-      <c r="H33" s="5">
-        <f>SUM(H2:H32)</f>
+    <row r="33" spans="6:9" x14ac:dyDescent="0.35">
+      <c r="F33" s="5">
+        <f>SUM(F2:F32)</f>
         <v>599907</v>
       </c>
     </row>
-    <row r="35" spans="8:11" x14ac:dyDescent="0.35">
-      <c r="K35" s="5"/>
+    <row r="35" spans="6:9" x14ac:dyDescent="0.35">
+      <c r="I35" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15424,533 +15402,527 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E3E60C9-7190-4A23-8149-6DE2F233D92A}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.90625" style="8" customWidth="1"/>
-    <col min="2" max="3" width="13" style="5" customWidth="1"/>
-    <col min="4" max="5" width="17.36328125" style="5" customWidth="1"/>
-    <col min="6" max="7" width="15.81640625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="14.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="15.81640625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>46054</v>
       </c>
+      <c r="B2" s="5">
+        <v>4900</v>
+      </c>
       <c r="C2" s="5">
-        <v>4900</v>
-      </c>
-      <c r="E2" s="5">
         <v>10500</v>
       </c>
+      <c r="D2" s="5">
+        <v>6000</v>
+      </c>
       <c r="F2" s="5">
-        <v>6000</v>
-      </c>
-      <c r="H2" s="5">
-        <f>SUM(B2:G2)</f>
+        <f>SUM(B2:E2)</f>
         <v>21400</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>46055</v>
       </c>
+      <c r="B3" s="5">
+        <v>7350</v>
+      </c>
       <c r="C3" s="5">
-        <v>7350</v>
-      </c>
-      <c r="E3" s="5">
         <f>830+170+8000</f>
         <v>9000</v>
       </c>
+      <c r="D3" s="5">
+        <v>6000</v>
+      </c>
       <c r="F3" s="5">
-        <v>6000</v>
-      </c>
-      <c r="H3" s="5">
-        <f t="shared" ref="H3:H29" si="0">SUM(B3:G3)</f>
+        <f>SUM(B3:E3)</f>
         <v>22350</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>46056</v>
       </c>
+      <c r="B4" s="5">
+        <v>10500</v>
+      </c>
       <c r="C4" s="5">
-        <v>10500</v>
-      </c>
-      <c r="E4" s="5">
         <v>6000</v>
       </c>
+      <c r="D4" s="5">
+        <v>4100</v>
+      </c>
       <c r="F4" s="5">
-        <v>4100</v>
-      </c>
-      <c r="H4" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B4:E4)</f>
         <v>20600</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>46057</v>
       </c>
+      <c r="B5" s="5">
+        <v>2900</v>
+      </c>
       <c r="C5" s="5">
-        <v>2900</v>
-      </c>
-      <c r="E5" s="5">
         <f>1188+10500</f>
         <v>11688</v>
       </c>
+      <c r="D5" s="5">
+        <v>3700</v>
+      </c>
       <c r="F5" s="5">
-        <v>3700</v>
-      </c>
-      <c r="H5" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B5:E5)</f>
         <v>18288</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>46058</v>
       </c>
+      <c r="B6" s="5">
+        <v>7600</v>
+      </c>
       <c r="C6" s="5">
-        <v>7600</v>
-      </c>
-      <c r="E6" s="5">
         <f>1414+210+400+4300</f>
         <v>6324</v>
       </c>
+      <c r="D6" s="5">
+        <v>6100</v>
+      </c>
       <c r="F6" s="5">
-        <v>6100</v>
-      </c>
-      <c r="H6" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B6:E6)</f>
         <v>20024</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>46059</v>
       </c>
+      <c r="B7" s="5">
+        <v>3500</v>
+      </c>
       <c r="C7" s="5">
-        <v>3500</v>
-      </c>
-      <c r="E7" s="5">
         <v>9000</v>
       </c>
+      <c r="D7" s="5">
+        <v>7800</v>
+      </c>
       <c r="F7" s="5">
-        <v>7800</v>
-      </c>
-      <c r="H7" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B7:E7)</f>
         <v>20300</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>46060</v>
       </c>
+      <c r="B8" s="5">
+        <v>9700</v>
+      </c>
       <c r="C8" s="5">
-        <v>9700</v>
-      </c>
-      <c r="E8" s="5">
         <v>5250</v>
       </c>
+      <c r="D8" s="5">
+        <v>6000</v>
+      </c>
       <c r="F8" s="5">
-        <v>6000</v>
-      </c>
-      <c r="H8" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B8:E8)</f>
         <v>20950</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>46061</v>
       </c>
+      <c r="B9" s="5">
+        <v>8800</v>
+      </c>
       <c r="C9" s="5">
-        <v>8800</v>
-      </c>
-      <c r="E9" s="5">
         <v>5900</v>
       </c>
+      <c r="D9" s="5">
+        <v>5000</v>
+      </c>
       <c r="F9" s="5">
-        <v>5000</v>
-      </c>
-      <c r="H9" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B9:E9)</f>
         <v>19700</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>46062</v>
       </c>
+      <c r="B10" s="5">
+        <v>12600</v>
+      </c>
       <c r="C10" s="5">
-        <v>12600</v>
-      </c>
-      <c r="E10" s="5">
         <v>7624</v>
       </c>
+      <c r="D10" s="5">
+        <v>7600</v>
+      </c>
       <c r="F10" s="5">
-        <v>7600</v>
-      </c>
-      <c r="H10" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B10:E10)</f>
         <v>27824</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46063</v>
       </c>
+      <c r="B11" s="5">
+        <v>11400</v>
+      </c>
       <c r="C11" s="5">
-        <v>11400</v>
-      </c>
-      <c r="E11" s="5">
         <v>6610</v>
       </c>
+      <c r="D11" s="5">
+        <v>5400</v>
+      </c>
       <c r="F11" s="5">
-        <v>5400</v>
-      </c>
-      <c r="H11" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B11:E11)</f>
         <v>23410</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>46064</v>
       </c>
+      <c r="B12" s="5">
+        <v>12200</v>
+      </c>
       <c r="C12" s="5">
-        <v>12200</v>
-      </c>
-      <c r="E12" s="5">
         <f>5700+210</f>
         <v>5910</v>
       </c>
+      <c r="D12" s="5">
+        <v>6500</v>
+      </c>
       <c r="F12" s="5">
-        <v>6500</v>
-      </c>
-      <c r="H12" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B12:E12)</f>
         <v>24610</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>46065</v>
       </c>
+      <c r="B13" s="5">
+        <v>14100</v>
+      </c>
       <c r="C13" s="5">
-        <v>14100</v>
-      </c>
-      <c r="E13" s="5">
         <v>4300</v>
       </c>
+      <c r="D13" s="5">
+        <v>6200</v>
+      </c>
       <c r="F13" s="5">
-        <v>6200</v>
-      </c>
-      <c r="H13" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B13:E13)</f>
         <v>24600</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>46066</v>
       </c>
+      <c r="B14" s="5">
+        <v>15800</v>
+      </c>
       <c r="C14" s="5">
-        <v>15800</v>
-      </c>
-      <c r="E14" s="5">
         <v>7700</v>
       </c>
+      <c r="D14" s="5">
+        <v>6800</v>
+      </c>
       <c r="F14" s="5">
-        <v>6800</v>
-      </c>
-      <c r="H14" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B14:E14)</f>
         <v>30300</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>46067</v>
       </c>
+      <c r="B15" s="5">
+        <v>13000</v>
+      </c>
       <c r="C15" s="5">
-        <v>13000</v>
-      </c>
-      <c r="E15" s="5">
         <v>6650</v>
       </c>
+      <c r="D15" s="5">
+        <v>4300</v>
+      </c>
       <c r="F15" s="5">
-        <v>4300</v>
-      </c>
-      <c r="H15" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B15:E15)</f>
         <v>23950</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>46068</v>
       </c>
+      <c r="B16" s="5">
+        <v>6900</v>
+      </c>
       <c r="C16" s="5">
-        <v>6900</v>
-      </c>
-      <c r="E16" s="5">
         <v>8800</v>
       </c>
+      <c r="D16" s="5">
+        <v>4200</v>
+      </c>
       <c r="F16" s="5">
-        <v>4200</v>
-      </c>
-      <c r="H16" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B16:E16)</f>
         <v>19900</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46069</v>
       </c>
+      <c r="B17" s="5">
+        <v>23000</v>
+      </c>
       <c r="C17" s="5">
-        <v>23000</v>
-      </c>
-      <c r="E17" s="5">
         <v>13500</v>
       </c>
+      <c r="D17" s="5">
+        <v>9800</v>
+      </c>
       <c r="F17" s="5">
-        <v>9800</v>
-      </c>
-      <c r="H17" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B17:E17)</f>
         <v>46300</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>46070</v>
       </c>
-      <c r="H18" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F18" s="5">
+        <f>SUM(B18:E18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>46071</v>
       </c>
-      <c r="H19" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F19" s="5">
+        <f>SUM(B19:E19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>46072</v>
       </c>
-      <c r="H20" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F20" s="5">
+        <f>SUM(B20:E20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>46073</v>
       </c>
+      <c r="B21" s="5">
+        <v>8300</v>
+      </c>
       <c r="C21" s="5">
-        <v>8300</v>
-      </c>
-      <c r="E21" s="5">
         <v>5700</v>
       </c>
+      <c r="D21" s="5">
+        <v>4500</v>
+      </c>
       <c r="F21" s="5">
-        <v>4500</v>
-      </c>
-      <c r="H21" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B21:E21)</f>
         <v>18500</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>46074</v>
       </c>
+      <c r="B22" s="5">
+        <v>10400</v>
+      </c>
       <c r="C22" s="5">
-        <v>10400</v>
-      </c>
-      <c r="E22" s="5">
         <v>4300</v>
       </c>
+      <c r="D22" s="5">
+        <v>2700</v>
+      </c>
       <c r="F22" s="5">
-        <v>2700</v>
-      </c>
-      <c r="H22" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B22:E22)</f>
         <v>17400</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>46075</v>
       </c>
+      <c r="B23" s="5">
+        <v>13000</v>
+      </c>
       <c r="C23" s="5">
-        <v>13000</v>
-      </c>
-      <c r="E23" s="5">
         <v>4700</v>
       </c>
+      <c r="D23" s="5">
+        <v>2800</v>
+      </c>
       <c r="F23" s="5">
-        <v>2800</v>
-      </c>
-      <c r="H23" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B23:E23)</f>
         <v>20500</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46076</v>
       </c>
+      <c r="B24" s="5">
+        <v>7450</v>
+      </c>
       <c r="C24" s="5">
-        <v>7450</v>
-      </c>
-      <c r="E24" s="5">
         <v>5500</v>
       </c>
+      <c r="D24" s="5">
+        <v>5900</v>
+      </c>
       <c r="F24" s="5">
-        <v>5900</v>
-      </c>
-      <c r="H24" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B24:E24)</f>
         <v>18850</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>46077</v>
       </c>
+      <c r="B25" s="5">
+        <v>10600</v>
+      </c>
       <c r="C25" s="5">
-        <v>10600</v>
-      </c>
-      <c r="E25" s="5">
         <v>6000</v>
       </c>
+      <c r="D25" s="5">
+        <v>5300</v>
+      </c>
       <c r="F25" s="5">
-        <v>5300</v>
-      </c>
-      <c r="H25" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B25:E25)</f>
         <v>21900</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>46078</v>
       </c>
+      <c r="B26" s="5">
+        <v>12730</v>
+      </c>
       <c r="C26" s="5">
-        <v>12730</v>
-      </c>
-      <c r="E26" s="5">
         <v>7000</v>
       </c>
+      <c r="D26" s="5">
+        <v>4100</v>
+      </c>
       <c r="F26" s="5">
-        <v>4100</v>
-      </c>
-      <c r="H26" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B26:E26)</f>
         <v>23830</v>
       </c>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>46079</v>
       </c>
+      <c r="B27" s="5">
+        <v>7550</v>
+      </c>
       <c r="C27" s="5">
-        <v>7550</v>
-      </c>
-      <c r="E27" s="5">
         <v>5500</v>
       </c>
+      <c r="D27" s="5">
+        <v>4200</v>
+      </c>
       <c r="F27" s="5">
-        <v>4200</v>
-      </c>
-      <c r="H27" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B27:E27)</f>
         <v>17250</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>46080</v>
       </c>
+      <c r="B28" s="5">
+        <v>10468</v>
+      </c>
       <c r="C28" s="5">
-        <v>10468</v>
-      </c>
-      <c r="E28" s="5">
         <v>5750</v>
       </c>
+      <c r="D28" s="5">
+        <v>2700</v>
+      </c>
       <c r="F28" s="5">
-        <v>2700</v>
-      </c>
-      <c r="H28" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B28:E28)</f>
         <v>18918</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>46081</v>
       </c>
+      <c r="B29" s="5">
+        <v>10500</v>
+      </c>
       <c r="C29" s="5">
-        <v>10500</v>
-      </c>
-      <c r="E29" s="5">
         <v>2300</v>
       </c>
+      <c r="D29" s="5">
+        <v>3900</v>
+      </c>
       <c r="F29" s="5">
-        <v>3900</v>
-      </c>
-      <c r="H29" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B29:E29)</f>
         <v>16700</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="H30" s="5">
-        <f>SUM(H2:H29)</f>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F30" s="5">
+        <f>SUM(F2:F29)</f>
         <v>558354</v>
       </c>
     </row>
-    <row r="35" spans="11:11" x14ac:dyDescent="0.35">
-      <c r="K35" s="5"/>
+    <row r="35" spans="9:9" x14ac:dyDescent="0.35">
+      <c r="I35" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15960,626 +15932,614 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D566CA81-9F1B-4B0B-AFE2-BB40F0C8C303}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.90625" style="8" customWidth="1"/>
-    <col min="2" max="3" width="13" style="5" customWidth="1"/>
-    <col min="4" max="5" width="17.36328125" style="5" customWidth="1"/>
-    <col min="6" max="7" width="15.81640625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="14.81640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="15.81640625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>46023</v>
       </c>
       <c r="B2" s="5">
-        <v>4850</v>
+        <v>5350</v>
       </c>
       <c r="C2" s="5">
-        <v>5350</v>
-      </c>
-      <c r="E2" s="5">
-        <v>3400</v>
+        <v>8300</v>
+      </c>
+      <c r="D2" s="5">
+        <v>9500</v>
       </c>
       <c r="F2" s="5">
-        <v>9500</v>
-      </c>
-      <c r="H2" s="5">
-        <f>SUM(B2:G2)</f>
-        <v>23100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <f>SUM(B2:E2)</f>
+        <v>23150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>46024</v>
       </c>
+      <c r="B3" s="5">
+        <v>6500</v>
+      </c>
       <c r="C3" s="5">
-        <v>6500</v>
-      </c>
-      <c r="E3" s="5">
         <v>5600</v>
       </c>
+      <c r="D3" s="5">
+        <v>3000</v>
+      </c>
       <c r="F3" s="5">
-        <v>3000</v>
-      </c>
-      <c r="H3" s="5">
-        <f t="shared" ref="H3:H32" si="0">SUM(B3:G3)</f>
+        <f>SUM(B3:E3)</f>
         <v>15100</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>46025</v>
       </c>
       <c r="B4" s="5">
-        <v>4700</v>
+        <v>4450</v>
       </c>
       <c r="C4" s="5">
-        <v>4450</v>
-      </c>
-      <c r="E4" s="5">
-        <v>3200</v>
+        <v>7900</v>
+      </c>
+      <c r="D4" s="5">
+        <v>7100</v>
       </c>
       <c r="F4" s="5">
-        <v>7100</v>
-      </c>
-      <c r="H4" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B4:E4)</f>
         <v>19450</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>46026</v>
       </c>
+      <c r="B5" s="5">
+        <v>6350</v>
+      </c>
       <c r="C5" s="5">
-        <v>6350</v>
-      </c>
-      <c r="E5" s="5">
         <v>6150</v>
       </c>
+      <c r="D5" s="5">
+        <v>4000</v>
+      </c>
       <c r="F5" s="5">
-        <v>4000</v>
-      </c>
-      <c r="H5" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B5:E5)</f>
         <v>16500</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>46027</v>
       </c>
+      <c r="B6" s="5">
+        <v>7800</v>
+      </c>
       <c r="C6" s="5">
-        <v>7800</v>
-      </c>
-      <c r="E6" s="5">
         <v>7450</v>
       </c>
+      <c r="D6" s="5">
+        <v>3300</v>
+      </c>
       <c r="F6" s="5">
-        <v>3300</v>
-      </c>
-      <c r="H6" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B6:E6)</f>
         <v>18550</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>46028</v>
       </c>
+      <c r="B7" s="5">
+        <v>9867</v>
+      </c>
       <c r="C7" s="5">
-        <v>9867</v>
-      </c>
-      <c r="E7" s="5">
         <v>3550</v>
       </c>
+      <c r="D7" s="5">
+        <v>5500</v>
+      </c>
       <c r="F7" s="5">
-        <v>5500</v>
-      </c>
-      <c r="H7" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B7:E7)</f>
         <v>18917</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>46029</v>
       </c>
+      <c r="B8" s="5">
+        <v>8500</v>
+      </c>
       <c r="C8" s="5">
-        <v>8500</v>
-      </c>
-      <c r="E8" s="5">
         <v>6500</v>
       </c>
+      <c r="D8" s="5">
+        <v>4590</v>
+      </c>
       <c r="F8" s="5">
-        <v>4590</v>
-      </c>
-      <c r="H8" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B8:E8)</f>
         <v>19590</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>46030</v>
       </c>
+      <c r="B9" s="5">
+        <v>7514</v>
+      </c>
       <c r="C9" s="5">
-        <v>7514</v>
-      </c>
-      <c r="E9" s="5">
         <v>6250</v>
       </c>
+      <c r="D9" s="5">
+        <v>4000</v>
+      </c>
       <c r="F9" s="5">
-        <v>4000</v>
-      </c>
-      <c r="H9" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B9:E9)</f>
         <v>17764</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>46031</v>
       </c>
+      <c r="B10" s="5">
+        <v>8200</v>
+      </c>
       <c r="C10" s="5">
-        <v>8200</v>
-      </c>
-      <c r="E10" s="5">
         <v>4350</v>
       </c>
+      <c r="D10" s="5">
+        <v>4222</v>
+      </c>
       <c r="F10" s="5">
-        <v>4222</v>
-      </c>
-      <c r="H10" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B10:E10)</f>
         <v>16772</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46032</v>
       </c>
+      <c r="B11" s="5">
+        <v>9250</v>
+      </c>
       <c r="C11" s="5">
-        <v>9250</v>
-      </c>
-      <c r="E11" s="5">
         <v>7000</v>
       </c>
+      <c r="D11" s="5">
+        <v>3800</v>
+      </c>
       <c r="F11" s="5">
-        <v>3800</v>
-      </c>
-      <c r="H11" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B11:E11)</f>
         <v>20050</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>46033</v>
       </c>
+      <c r="B12" s="5">
+        <v>8550</v>
+      </c>
       <c r="C12" s="5">
-        <v>8550</v>
-      </c>
-      <c r="E12" s="5">
         <v>3250</v>
       </c>
+      <c r="D12" s="5">
+        <v>3400</v>
+      </c>
       <c r="F12" s="5">
-        <v>3400</v>
-      </c>
-      <c r="H12" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B12:E12)</f>
         <v>15200</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>46034</v>
       </c>
+      <c r="B13" s="5">
+        <v>10900</v>
+      </c>
       <c r="C13" s="5">
-        <v>10900</v>
-      </c>
-      <c r="E13" s="5">
         <v>7050</v>
       </c>
+      <c r="D13" s="5">
+        <v>6300</v>
+      </c>
       <c r="F13" s="5">
-        <v>6300</v>
-      </c>
-      <c r="H13" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B13:E13)</f>
         <v>24250</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>46035</v>
       </c>
+      <c r="B14" s="5">
+        <v>11150</v>
+      </c>
       <c r="C14" s="5">
-        <v>11150</v>
-      </c>
-      <c r="E14" s="5">
         <v>6600</v>
       </c>
+      <c r="D14" s="5">
+        <v>5900</v>
+      </c>
       <c r="F14" s="5">
-        <v>5900</v>
-      </c>
-      <c r="H14" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B14:E14)</f>
         <v>23650</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>46036</v>
       </c>
+      <c r="B15" s="5">
+        <v>13200</v>
+      </c>
       <c r="C15" s="5">
-        <v>13200</v>
-      </c>
-      <c r="E15" s="5">
         <v>4300</v>
       </c>
+      <c r="D15" s="5">
+        <v>3500</v>
+      </c>
       <c r="F15" s="5">
-        <v>3500</v>
-      </c>
-      <c r="H15" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B15:E15)</f>
         <v>21000</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>46037</v>
       </c>
+      <c r="B16" s="5">
+        <v>11600</v>
+      </c>
       <c r="C16" s="5">
-        <v>11600</v>
-      </c>
-      <c r="E16" s="5">
         <v>4200</v>
       </c>
+      <c r="D16" s="5">
+        <v>2490</v>
+      </c>
       <c r="F16" s="5">
-        <v>2490</v>
-      </c>
-      <c r="H16" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B16:E16)</f>
         <v>18290</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46038</v>
       </c>
+      <c r="B17" s="5">
+        <v>13000</v>
+      </c>
       <c r="C17" s="5">
-        <v>13000</v>
-      </c>
-      <c r="E17" s="5">
         <v>6300</v>
       </c>
+      <c r="D17" s="5">
+        <v>5600</v>
+      </c>
       <c r="F17" s="5">
-        <v>5600</v>
-      </c>
-      <c r="H17" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B17:E17)</f>
         <v>24900</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>46039</v>
       </c>
+      <c r="B18" s="5">
+        <v>8300</v>
+      </c>
       <c r="C18" s="5">
-        <v>8300</v>
-      </c>
-      <c r="E18" s="5">
         <v>5200</v>
       </c>
+      <c r="D18" s="5">
+        <v>7400</v>
+      </c>
       <c r="F18" s="5">
-        <v>7400</v>
-      </c>
-      <c r="H18" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B18:E18)</f>
         <v>20900</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>46040</v>
       </c>
+      <c r="B19" s="5">
+        <v>7900</v>
+      </c>
       <c r="C19" s="5">
-        <v>7900</v>
-      </c>
-      <c r="E19" s="5">
         <v>4100</v>
       </c>
+      <c r="D19" s="5">
+        <v>5200</v>
+      </c>
       <c r="F19" s="5">
-        <v>5200</v>
-      </c>
-      <c r="H19" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B19:E19)</f>
         <v>17200</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>46041</v>
       </c>
+      <c r="B20" s="5">
+        <v>8580</v>
+      </c>
       <c r="C20" s="5">
-        <v>8580</v>
-      </c>
-      <c r="E20" s="5">
         <v>5100</v>
       </c>
+      <c r="D20" s="5">
+        <v>10100</v>
+      </c>
       <c r="F20" s="5">
-        <v>10100</v>
-      </c>
-      <c r="H20" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B20:E20)</f>
         <v>23780</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>46042</v>
       </c>
+      <c r="B21" s="5">
+        <v>11150</v>
+      </c>
       <c r="C21" s="5">
-        <v>11150</v>
-      </c>
-      <c r="E21" s="5">
         <v>4800</v>
       </c>
+      <c r="D21" s="5">
+        <v>3400</v>
+      </c>
       <c r="F21" s="5">
-        <v>3400</v>
-      </c>
-      <c r="H21" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B21:E21)</f>
         <v>19350</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>46043</v>
       </c>
+      <c r="B22" s="5">
+        <v>10100</v>
+      </c>
       <c r="C22" s="5">
-        <v>10100</v>
-      </c>
-      <c r="E22" s="5">
         <v>3550</v>
       </c>
+      <c r="D22" s="5">
+        <v>5300</v>
+      </c>
       <c r="F22" s="5">
-        <v>5300</v>
-      </c>
-      <c r="H22" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B22:E22)</f>
         <v>18950</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>46044</v>
       </c>
+      <c r="B23" s="5">
+        <v>10500</v>
+      </c>
       <c r="C23" s="5">
-        <v>10500</v>
-      </c>
-      <c r="E23" s="5">
         <v>6100</v>
       </c>
+      <c r="D23" s="5">
+        <v>4500</v>
+      </c>
       <c r="F23" s="5">
-        <v>4500</v>
-      </c>
-      <c r="H23" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B23:E23)</f>
         <v>21100</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46045</v>
       </c>
+      <c r="B24" s="5">
+        <v>7300</v>
+      </c>
       <c r="C24" s="5">
-        <v>7300</v>
-      </c>
-      <c r="E24" s="5">
         <v>5800</v>
       </c>
+      <c r="D24" s="5">
+        <v>4000</v>
+      </c>
       <c r="F24" s="5">
-        <v>4000</v>
-      </c>
-      <c r="H24" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B24:E24)</f>
         <v>17100</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>46046</v>
       </c>
+      <c r="B25" s="5">
+        <v>10200</v>
+      </c>
       <c r="C25" s="5">
-        <v>10200</v>
-      </c>
-      <c r="E25" s="5">
         <v>3400</v>
       </c>
+      <c r="D25" s="5">
+        <v>5800</v>
+      </c>
       <c r="F25" s="5">
-        <v>5800</v>
-      </c>
-      <c r="H25" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B25:E25)</f>
         <v>19400</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>46047</v>
       </c>
+      <c r="B26" s="5">
+        <v>13600</v>
+      </c>
       <c r="C26" s="5">
-        <v>13600</v>
-      </c>
-      <c r="E26" s="5">
         <v>2500</v>
       </c>
+      <c r="D26" s="5">
+        <v>6300</v>
+      </c>
       <c r="F26" s="5">
-        <v>6300</v>
-      </c>
-      <c r="H26" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B26:E26)</f>
         <v>22400</v>
       </c>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>46048</v>
       </c>
+      <c r="B27" s="5">
+        <v>9600</v>
+      </c>
       <c r="C27" s="5">
-        <v>9600</v>
-      </c>
-      <c r="E27" s="5">
         <f>1088+5500</f>
         <v>6588</v>
       </c>
+      <c r="D27" s="5">
+        <v>4200</v>
+      </c>
       <c r="F27" s="5">
-        <v>4200</v>
-      </c>
-      <c r="H27" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B27:E27)</f>
         <v>20388</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>46049</v>
       </c>
+      <c r="B28" s="5">
+        <v>11300</v>
+      </c>
       <c r="C28" s="5">
-        <v>11300</v>
-      </c>
-      <c r="E28" s="5">
         <f>238+5700</f>
         <v>5938</v>
       </c>
+      <c r="D28" s="5">
+        <v>8100</v>
+      </c>
       <c r="F28" s="5">
-        <v>8100</v>
-      </c>
-      <c r="H28" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B28:E28)</f>
         <v>25338</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>46050</v>
       </c>
+      <c r="B29" s="5">
+        <v>10800</v>
+      </c>
       <c r="C29" s="5">
-        <v>10800</v>
-      </c>
-      <c r="E29" s="5">
         <v>7300</v>
       </c>
+      <c r="D29" s="5">
+        <v>4300</v>
+      </c>
       <c r="F29" s="5">
-        <v>4300</v>
-      </c>
-      <c r="H29" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B29:E29)</f>
         <v>22400</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>46051</v>
       </c>
+      <c r="B30" s="5">
+        <v>6800</v>
+      </c>
       <c r="C30" s="5">
-        <v>6800</v>
-      </c>
-      <c r="E30" s="5">
         <f>1310+475+8700</f>
         <v>10485</v>
       </c>
+      <c r="D30" s="5">
+        <v>5000</v>
+      </c>
       <c r="F30" s="5">
-        <v>5000</v>
-      </c>
-      <c r="H30" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B30:E30)</f>
         <v>22285</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>46052</v>
       </c>
+      <c r="B31" s="5">
+        <v>13300</v>
+      </c>
       <c r="C31" s="5">
-        <v>13300</v>
-      </c>
-      <c r="E31" s="5">
         <f>205+6400</f>
         <v>6605</v>
       </c>
+      <c r="D31" s="5">
+        <v>4000</v>
+      </c>
       <c r="F31" s="5">
-        <v>4000</v>
-      </c>
-      <c r="H31" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B31:E31)</f>
         <v>23905</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>46053</v>
       </c>
+      <c r="B32" s="5">
+        <v>12800</v>
+      </c>
       <c r="C32" s="5">
-        <v>12800</v>
-      </c>
-      <c r="E32" s="5">
         <v>4000</v>
       </c>
+      <c r="D32" s="5">
+        <v>10000</v>
+      </c>
       <c r="F32" s="5">
-        <v>10000</v>
-      </c>
-      <c r="H32" s="5">
-        <f t="shared" si="0"/>
+        <f>SUM(B32:E32)</f>
         <v>26800</v>
       </c>
     </row>
-    <row r="33" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="H33" s="5">
-        <f>SUM(H2:H32)</f>
-        <v>634379</v>
-      </c>
-    </row>
-    <row r="35" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="F35" s="5">
+    <row r="33" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="F33" s="5">
         <f>SUM(F2:F32)</f>
+        <v>634429</v>
+      </c>
+    </row>
+    <row r="35" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="D35" s="5">
+        <f>SUM(D2:D32)</f>
         <v>163802</v>
       </c>
     </row>
-    <row r="37" spans="6:11" x14ac:dyDescent="0.35">
-      <c r="K37" s="5"/>
+    <row r="37" spans="4:9" x14ac:dyDescent="0.35">
+      <c r="I37" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>